<commit_message>
push button added; IMU updated
</commit_message>
<xml_diff>
--- a/BoM_overall.xlsx
+++ b/BoM_overall.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PhantomKid\OneDrive - Imperial College London\Desktop\FPSP_Camera_FPC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB61CB4-A64C-4289-90C5-E701A42AFCBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10136908-FE3C-4AF5-8C26-3BDD171ACCC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="52">
   <si>
     <t>Part Name</t>
   </si>
@@ -36,9 +36,6 @@
     <t>USB_B_Micro</t>
   </si>
   <si>
-    <t>Conn_02x04_Counter_Clockwise</t>
-  </si>
-  <si>
     <t>Conn_02x07_Counter_Clockwise</t>
   </si>
   <si>
@@ -51,9 +48,6 @@
     <t>IMU</t>
   </si>
   <si>
-    <t>ICM-45686</t>
-  </si>
-  <si>
     <t>LDO</t>
   </si>
   <si>
@@ -69,18 +63,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Molex_SlimStack_502430-0822_2x04_P0.40mm_Vertical</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>https://uk.farnell.com/tdk/icm-45686/mems-module-6-axis-1-71v-3-6v/dp/4572492</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>https://uk.farnell.com/jst-japan-solderless-terminals/sm03b-srss-tb-lf-sn/header-r-a-3way/dp/1679118</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Quantity</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -125,14 +111,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>https://www.mouser.co.uk/ProductDetail/Molex/502430-0822?qs=byeeYqUIh0ORWNduRUQWFQ%3D%3D</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Molex_SlimStack_502426-0812_2x04_P0.40mm_Vertical</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Source</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -149,10 +127,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>https://www.mouser.co.uk/ProductDetail/Molex/502426-0812?qs=byeeYqUIh0O%252BW14PukUHXw%3D%3D</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>https://www.mouser.co.uk/ProductDetail/Texas-Instruments/TLV73315PQDRVRQ1?qs=Euq2YPj5ArIsMkihzFWY8w%3D%3D</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -193,12 +167,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>538-50243-00822</t>
-  </si>
-  <si>
-    <t>538-50242-60812</t>
-  </si>
-  <si>
     <t>595-TLV73315PQDRVRQ1</t>
   </si>
   <si>
@@ -217,6 +185,41 @@
   </si>
   <si>
     <t>Order Code / Mouser No</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>LSM6DSLTR</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://uk.farnell.com/stmicroelectronics/lsm6dsltr/inemo-inertial-module-2-4-8-16g/dp/2761748</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Switch (slide)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CAS-120TA1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://uk.farnell.com/nidec-copal-electronics/cas-120ta/slide-switch-spdt-0-1a-6vdc-smd/dp/2854716</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Push Button</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://www.mouser.co.uk/ProductDetail/CK/PTS526SM15SMTR2-LFS?qs=Imq1NPwxi75LpUh6FiCy2w%3D%3D</t>
+  </si>
+  <si>
+    <t>611-PTS526SM15SMTR2L</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PTS526SM15SMTR2 LFS</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -640,19 +643,19 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="16" x14ac:dyDescent="0.3">
@@ -660,13 +663,13 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C2" s="6">
         <v>5</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E2" s="6">
         <v>1.2</v>
@@ -675,7 +678,7 @@
         <v>1568026</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="16" x14ac:dyDescent="0.3">
@@ -683,36 +686,36 @@
         <v>3</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="C3" s="6">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E3" s="6">
-        <v>0.52</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>27</v>
+        <v>0.86799999999999999</v>
+      </c>
+      <c r="F3" s="6">
+        <v>3500584</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="16" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="C4" s="6">
         <v>10</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E4" s="6">
         <v>0.46500000000000002</v>
@@ -721,67 +724,67 @@
         <v>3911710</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="16" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>3</v>
+        <v>45</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="C5" s="6">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E5" s="6">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>45</v>
+        <v>1.1832</v>
+      </c>
+      <c r="F5" s="6">
+        <v>2854716</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="16" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>4</v>
+        <v>48</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>35</v>
+        <v>51</v>
       </c>
       <c r="C6" s="6">
         <v>10</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E6" s="6">
-        <v>0.86799999999999999</v>
-      </c>
-      <c r="F6" s="6">
-        <v>3500584</v>
+        <v>0.12</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>50</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="16" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>5</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>6</v>
       </c>
       <c r="C7" s="6">
         <v>5</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E7" s="6">
         <v>0.52</v>
@@ -790,21 +793,21 @@
         <v>1679118</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>15</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="16" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>8</v>
+        <v>43</v>
       </c>
       <c r="C8" s="6">
         <v>5</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E8" s="6">
         <v>7.8840000000000003</v>
@@ -813,90 +816,90 @@
         <v>4572492</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="16" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C9" s="6">
         <v>5</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E9" s="6">
         <v>0.44</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="16" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C10" s="6">
         <v>5</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E10" s="6">
         <v>0.751</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="16" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C11" s="6">
         <v>5</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E11" s="6">
         <v>0.72099999999999997</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="16" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="C12" s="6">
         <v>10</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E12" s="6">
         <v>2.3519999999999999</v>
@@ -905,57 +908,57 @@
         <v>2396220</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="154" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="C13" s="6">
         <v>2</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="16" x14ac:dyDescent="0.3">
       <c r="A15" s="8" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="16" x14ac:dyDescent="0.3">
       <c r="A16" s="8" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="G2" r:id="rId1" xr:uid="{7629E2FA-41F2-4CC2-B4D7-BFE323D6BFEE}"/>
-    <hyperlink ref="G8" r:id="rId2" xr:uid="{EB753440-38A8-4DA6-833C-8FBBF56BA123}"/>
-    <hyperlink ref="G7" r:id="rId3" xr:uid="{BFE6737D-6A99-48C9-9EEC-0FB628B3B520}"/>
-    <hyperlink ref="G10" r:id="rId4" xr:uid="{E9A01CE4-0A4B-482F-90F9-693C763BCC26}"/>
-    <hyperlink ref="G11" r:id="rId5" xr:uid="{A68F70EA-E132-45B6-88B9-7DA499D5151E}"/>
-    <hyperlink ref="G3" r:id="rId6" xr:uid="{AEBBA3C6-82D7-4357-A655-56F80275F8A2}"/>
-    <hyperlink ref="G5" r:id="rId7" xr:uid="{6C3E8ECD-7748-4996-82D2-BA98D65ABD1D}"/>
-    <hyperlink ref="G9" r:id="rId8" xr:uid="{8641ADBC-8FD0-4143-AC54-21678E95A300}"/>
-    <hyperlink ref="G4" r:id="rId9" xr:uid="{FBA0B1CC-FBAF-460B-A802-A017D365AA98}"/>
-    <hyperlink ref="G6" r:id="rId10" xr:uid="{C4D79EFD-DB3D-4D70-A982-81E289BF5310}"/>
-    <hyperlink ref="G12" r:id="rId11" xr:uid="{9C74FC71-0147-4849-808A-26A4DB3F8FF8}"/>
+    <hyperlink ref="G10" r:id="rId2" xr:uid="{E9A01CE4-0A4B-482F-90F9-693C763BCC26}"/>
+    <hyperlink ref="G11" r:id="rId3" xr:uid="{A68F70EA-E132-45B6-88B9-7DA499D5151E}"/>
+    <hyperlink ref="G9" r:id="rId4" xr:uid="{8641ADBC-8FD0-4143-AC54-21678E95A300}"/>
+    <hyperlink ref="G12" r:id="rId5" xr:uid="{9C74FC71-0147-4849-808A-26A4DB3F8FF8}"/>
+    <hyperlink ref="G8" r:id="rId6" xr:uid="{EB753440-38A8-4DA6-833C-8FBBF56BA123}"/>
+    <hyperlink ref="G4" r:id="rId7" xr:uid="{FBA0B1CC-FBAF-460B-A802-A017D365AA98}"/>
+    <hyperlink ref="G3" r:id="rId8" xr:uid="{8759A436-98A8-46D5-A008-2AE3F89907F9}"/>
+    <hyperlink ref="G7" r:id="rId9" xr:uid="{91BDEF6C-3932-4DF6-A566-1608E0996F2B}"/>
+    <hyperlink ref="G5" r:id="rId10" xr:uid="{2CD515ED-FCDA-4596-977D-7F804DCC3117}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId11"/>
 </worksheet>
 </file>
</xml_diff>